<commit_message>
Update cover letter with author information, revise page count in README and checklist, and correct geographic coverage details in systematic review documents. Adjustments reflect accurate authorship and enhance clarity on research gaps.
</commit_message>
<xml_diff>
--- a/JES_submission/Supplementary/quality_assessment.xlsx
+++ b/JES_submission/Supplementary/quality_assessment.xlsx
@@ -507,16 +507,16 @@
         <v>2007</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E2" s="2" t="n">
         <v>2</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -588,7 +588,7 @@
         <v>2014</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>1</v>
@@ -597,7 +597,7 @@
         <v>1</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
@@ -615,7 +615,7 @@
         <v>2015</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" s="2" t="n">
         <v>2</v>
@@ -624,7 +624,7 @@
         <v>1</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -858,7 +858,7 @@
         <v>2018</v>
       </c>
       <c r="D15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>1</v>
@@ -867,7 +867,7 @@
         <v>2</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16">
@@ -966,7 +966,7 @@
         <v>2019</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>1</v>
@@ -975,7 +975,7 @@
         <v>2</v>
       </c>
       <c r="G19" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20">
@@ -993,7 +993,7 @@
         <v>2019</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>1</v>
@@ -1002,7 +1002,7 @@
         <v>1</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="21">
@@ -1053,10 +1053,10 @@
         <v>1</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23">
@@ -1080,10 +1080,10 @@
         <v>1</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24">
@@ -1128,7 +1128,7 @@
         <v>2020</v>
       </c>
       <c r="D25" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="2" t="n">
         <v>1</v>
@@ -1137,7 +1137,7 @@
         <v>2</v>
       </c>
       <c r="G25" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26">
@@ -1209,7 +1209,7 @@
         <v>2020</v>
       </c>
       <c r="D28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E28" s="2" t="n">
         <v>1</v>
@@ -1218,7 +1218,7 @@
         <v>2</v>
       </c>
       <c r="G28" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29">
@@ -1236,13 +1236,13 @@
         <v>2021</v>
       </c>
       <c r="D29" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>4</v>
@@ -1263,7 +1263,7 @@
         <v>2021</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E30" s="2" t="n">
         <v>1</v>
@@ -1272,7 +1272,7 @@
         <v>1</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="31">
@@ -1290,13 +1290,13 @@
         <v>2021</v>
       </c>
       <c r="D31" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E31" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>4</v>
@@ -1317,7 +1317,7 @@
         <v>2021</v>
       </c>
       <c r="D32" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E32" s="2" t="n">
         <v>2</v>
@@ -1326,7 +1326,7 @@
         <v>1</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33">
@@ -1350,10 +1350,10 @@
         <v>1</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="34">
@@ -1377,10 +1377,10 @@
         <v>1</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
@@ -1458,10 +1458,10 @@
         <v>2</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="38">
@@ -1539,10 +1539,10 @@
         <v>1</v>
       </c>
       <c r="F40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="41">
@@ -1620,10 +1620,10 @@
         <v>2</v>
       </c>
       <c r="F43" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
@@ -1641,7 +1641,7 @@
         <v>2023</v>
       </c>
       <c r="D44" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>1</v>
@@ -1650,7 +1650,7 @@
         <v>1</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="45">
@@ -1722,7 +1722,7 @@
         <v>2023</v>
       </c>
       <c r="D47" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>1</v>
@@ -1731,7 +1731,7 @@
         <v>1</v>
       </c>
       <c r="G47" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="48">
@@ -1749,16 +1749,16 @@
         <v>2023</v>
       </c>
       <c r="D48" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G48" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="49">
@@ -1803,7 +1803,7 @@
         <v>2024</v>
       </c>
       <c r="D50" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>2</v>
@@ -1812,7 +1812,7 @@
         <v>1</v>
       </c>
       <c r="G50" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="51">
@@ -2025,10 +2025,10 @@
         <v>1</v>
       </c>
       <c r="F58" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="59">
@@ -2052,10 +2052,10 @@
         <v>1</v>
       </c>
       <c r="F59" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="60">
@@ -2133,10 +2133,10 @@
         <v>1</v>
       </c>
       <c r="F62" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="63">
@@ -2268,12 +2268,13 @@
         <v>1</v>
       </c>
       <c r="F67" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>3</v>
-      </c>
-    </row>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="68"/>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
@@ -2321,6 +2322,7 @@
         <v>6</v>
       </c>
     </row>
+    <row r="74"/>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
@@ -2365,7 +2367,7 @@
         </is>
       </c>
       <c r="B79" s="2" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="80">
@@ -2375,7 +2377,7 @@
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>29</v>
+        <v>41</v>
       </c>
     </row>
     <row r="81">
@@ -2385,7 +2387,7 @@
         </is>
       </c>
       <c r="B81" s="2" t="n">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="82">
@@ -2395,7 +2397,7 @@
         </is>
       </c>
       <c r="B82" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83">
@@ -2408,6 +2410,7 @@
         <v>0</v>
       </c>
     </row>
+    <row r="84"/>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
@@ -2422,7 +2425,7 @@
         </is>
       </c>
       <c r="B86" t="n">
-        <v>0.84</v>
+        <v>0.89</v>
       </c>
     </row>
     <row r="87">
@@ -2432,9 +2435,10 @@
         </is>
       </c>
       <c r="B87" t="n">
-        <v>1.11</v>
-      </c>
-    </row>
+        <v>1.38</v>
+      </c>
+    </row>
+    <row r="88"/>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
@@ -2447,7 +2451,7 @@
         <v>2007</v>
       </c>
       <c r="B90" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="91">
@@ -2463,7 +2467,7 @@
         <v>2014</v>
       </c>
       <c r="B92" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="93">
@@ -2471,7 +2475,7 @@
         <v>2015</v>
       </c>
       <c r="B93" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="94">
@@ -2503,7 +2507,7 @@
         <v>2019</v>
       </c>
       <c r="B97" s="2" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="98">
@@ -2511,7 +2515,7 @@
         <v>2020</v>
       </c>
       <c r="B98" s="2" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="99">
@@ -2535,7 +2539,7 @@
         <v>2023</v>
       </c>
       <c r="B101" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="102">

</xml_diff>